<commit_message>
Add long PDF retrieval and reranking pipeline
</commit_message>
<xml_diff>
--- a/reports/eval_met.xlsx
+++ b/reports/eval_met.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="eval_met" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eval_met" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'eval_met'!$A$1:$AK$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'eval_met'!$A$1:$AK$16</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK15"/>
+  <dimension ref="A1:AK16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="2"/>
@@ -2017,8 +2017,128 @@
         <v>0.02249982208013535</v>
       </c>
     </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-12T03:40:26Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Phase 0 live Groq smoke test</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>What does a solar panel convert into electricity?</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>140</v>
+      </c>
+      <c r="G16" t="n">
+        <v>131</v>
+      </c>
+      <c r="H16" t="n">
+        <v>9</v>
+      </c>
+      <c r="I16" s="1" t="n">
+        <v>6.428571428571428</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>0.3104005008935928</v>
+      </c>
+      <c r="L16" s="1" t="n">
+        <v>988.9636998996139</v>
+      </c>
+      <c r="M16" s="1" t="n">
+        <v>847.7598000317812</v>
+      </c>
+      <c r="N16" s="1" t="n">
+        <v>988.9636998996139</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>848.0702005326748</v>
+      </c>
+      <c r="P16" s="1" t="n">
+        <v>140.8934993669391</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>53</v>
+      </c>
+      <c r="R16" t="n">
+        <v>66</v>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Solar panels convert **sunlight** into electricity.</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>A solar panel converts sunlight into electricity.</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>Solar panels convert sunlight into electricity.</t>
+        </is>
+      </c>
+      <c r="V16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W16" s="1" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+      <c r="X16" s="3" t="n"/>
+      <c r="Y16" s="3" t="n"/>
+      <c r="Z16" s="1" t="n"/>
+      <c r="AA16" s="1" t="n"/>
+      <c r="AB16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="AE16" s="7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AF16" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI16" s="1" t="n">
+        <v>0.07360056042671204</v>
+      </c>
+      <c r="AJ16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" s="1" t="n">
+        <v>0.00360049307346344</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AK15"/>
+  <autoFilter ref="A1:AK16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clean HF metadata and configure Dockerfile for Render deployment
</commit_message>
<xml_diff>
--- a/reports/eval_met.xlsx
+++ b/reports/eval_met.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eval_met" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="eval_met" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'eval_met'!$A$1:$AK$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'eval_met'!$A$1:$AK$24</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK16"/>
+  <dimension ref="A1:AK24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="2"/>
@@ -2137,8 +2137,895 @@
         <v>0.00360049307346344</v>
       </c>
     </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-12T06:51:04Z</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>What are the dimensions for d_model, d_k, d_v, and the number of attention heads (h) used in the Transformer base model?</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G17" t="n">
+        <v>235</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2803</v>
+      </c>
+      <c r="I17" s="1" t="n">
+        <v>92.2646477946017</v>
+      </c>
+      <c r="J17" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>24675.2543002367</v>
+      </c>
+      <c r="L17" s="1" t="n">
+        <v>2003.115200437605</v>
+      </c>
+      <c r="M17" s="1" t="n">
+        <v>1025.49790032208</v>
+      </c>
+      <c r="N17" s="1" t="n">
+        <v>2003.115200437605</v>
+      </c>
+      <c r="O17" s="1" t="n">
+        <v>25700.75220055878</v>
+      </c>
+      <c r="P17" s="1" t="n">
+        <v>-23697.63700012118</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>409</v>
+      </c>
+      <c r="R17" t="n">
+        <v>129</v>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>The context states that the model uses **8 parallel attention heads (h = 8)**, and for each head the key and value dimensions are set to  
+- **dₖ = dᵥ = d_model / h = 64**.  
+Thus the overall model dimension is  
+- **d_model = h × 64 = 8 × 64 = 512**.  
+So, in the Transformer base model:  
+- **d_model = 512**  
+- **d_k = 64**  
+- **d_v = 64**  
+- **Number of attention heads (h) = 8**.</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain information about the specific dimensions \(d_{\text{model}}\), \(d_k\), \(d_v\) or the number of attention heads \(h\) used in the Transformer base model.</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr"/>
+      <c r="V17" s="1" t="n"/>
+      <c r="W17" s="1" t="n"/>
+      <c r="X17" s="3" t="n"/>
+      <c r="Y17" s="3" t="n"/>
+      <c r="Z17" s="1" t="n"/>
+      <c r="AA17" s="1" t="n"/>
+      <c r="AB17" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE17" s="7" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="AF17" s="7" t="n">
+        <v>0.3440000000000001</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH17" s="3" t="inlineStr">
+        <is>
+          <t>0,1,2,3,4,5</t>
+        </is>
+      </c>
+      <c r="AI17" s="1" t="n">
+        <v>17798.70809987187</v>
+      </c>
+      <c r="AJ17" s="1" t="n">
+        <v>6870.956600643694</v>
+      </c>
+      <c r="AK17" s="1" t="n">
+        <v>0.183500349521637</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-12T08:37:41Z</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>What are the dimensions for d_model, d_k, d_v, and the number of attention heads (h) used in the Transformer base model?</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3037</v>
+      </c>
+      <c r="G18" t="n">
+        <v>329</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2708</v>
+      </c>
+      <c r="I18" s="1" t="n">
+        <v>89.16694106025683</v>
+      </c>
+      <c r="J18" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>33759.5458002761</v>
+      </c>
+      <c r="L18" s="1" t="n">
+        <v>1777.788099832833</v>
+      </c>
+      <c r="M18" s="1" t="n">
+        <v>1195.338100194931</v>
+      </c>
+      <c r="N18" s="1" t="n">
+        <v>1777.788099832833</v>
+      </c>
+      <c r="O18" s="1" t="n">
+        <v>34954.88390047103</v>
+      </c>
+      <c r="P18" s="1" t="n">
+        <v>-33177.0958006382</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>285</v>
+      </c>
+      <c r="R18" t="n">
+        <v>186</v>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>The Transformer base model uses  
+- **d model = 512** (the overall model dimension)  
+- **d k = d v = 64** (the dimensions of each head’s keys and values)  
+- **h = 8** attention heads  
+These values are given in the text: “we employ h = 8 parallel attention layers… for each of these we use dk = dv = dmodel / h = 64,” and the model’s sub‑layers all produce outputs of dimension dmodel = 512.</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>The provided context only states that the model uses h = 8 parallel attention heads. It does not give the specific values for d_model, d_k, or d_v used in the Transformer base model. Therefore, the context does not contain enough information to answer that part of the question.</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr"/>
+      <c r="V18" s="1" t="n"/>
+      <c r="W18" s="1" t="n"/>
+      <c r="X18" s="3" t="n"/>
+      <c r="Y18" s="3" t="n"/>
+      <c r="Z18" s="1" t="n"/>
+      <c r="AA18" s="1" t="n"/>
+      <c r="AB18" s="7" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE18" s="7" t="n">
+        <v>0.516</v>
+      </c>
+      <c r="AF18" s="7" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="3" t="inlineStr">
+        <is>
+          <t>4,7,12,39,44,97</t>
+        </is>
+      </c>
+      <c r="AI18" s="1" t="n">
+        <v>17238.8971997425</v>
+      </c>
+      <c r="AJ18" s="1" t="n">
+        <v>16502.53930035979</v>
+      </c>
+      <c r="AK18" s="1" t="n">
+        <v>0.1670001074671745</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-12T08:39:06Z</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>How does scaled dot-product attention differ from additive attention, and why is the scaling factor 1/sqrt(d_k) applied?"</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>7</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G19" t="n">
+        <v>303</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2735</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>90.02633311389073</v>
+      </c>
+      <c r="J19" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>30941.79790001363</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>2353.812600485981</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>1490.284699946642</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>2353.812600485981</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>32432.08259996027</v>
+      </c>
+      <c r="P19" s="1" t="n">
+        <v>-30078.26999947429</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>620</v>
+      </c>
+      <c r="R19" t="n">
+        <v>147</v>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>**Scaled dot‑product attention vs. additive attention**
+- **Additive attention** computes the compatibility between a query \(q\) and a key \(k\) with a small feed‑forward network (one hidden layer). The result of that network is used as the score that is fed to the softmax.
+- **Scaled dot‑product (multiplicative) attention** computes the compatibility simply as the dot product \(q \cdot k\). All queries, keys and values are packed into matrices, so the whole operation can be performed with a single matrix multiplication, which makes it much faster and more memory‑efficient than the additive version.
+**Why the scaling factor \(1/\sqrt{d_k}\) is used**
+- When the dimensionality of the queries/keys \(d_k\) is large, the raw dot products have a variance that grows with \(d_k\) (the dot product of two random vectors of variance 1 has variance \(d_k\)).  
+- Large‑magnitude scores push the softmax into regions where its gradients are extremely small, hurting learning.  
+- Dividing the dot products by \(\sqrt{d_k}\) normalizes their magnitude, keeping the softmax inputs in a range where gradients remain healthy.  
+Thus, scaled dot‑product attention differs from additive attention in the way the compatibility function is computed (simple dot product vs. a learned feed‑forward network), and the factor \(1/\sqrt{d_k}\) is applied to stabilize training by preventing the dot‑product scores from becoming too large when \(d_k\) is large.</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain information about how scaled dot‑product attention differs from additive attention, nor does it explain why the scaling factor \(1/\sqrt{d_k}\) is used.</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr"/>
+      <c r="V19" s="1" t="n"/>
+      <c r="W19" s="1" t="n"/>
+      <c r="X19" s="3" t="n"/>
+      <c r="Y19" s="3" t="n"/>
+      <c r="Z19" s="1" t="n"/>
+      <c r="AA19" s="1" t="n"/>
+      <c r="AB19" s="7" t="n">
+        <v>0.7200000000000001</v>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE19" s="7" t="n">
+        <v>0.4259999999999999</v>
+      </c>
+      <c r="AF19" s="7" t="n">
+        <v>0.6320000000000001</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="3" t="inlineStr">
+        <is>
+          <t>68,69,93,98,119,122</t>
+        </is>
+      </c>
+      <c r="AI19" s="1" t="n">
+        <v>15178.3645004034</v>
+      </c>
+      <c r="AJ19" s="1" t="n">
+        <v>15749.54729992896</v>
+      </c>
+      <c r="AK19" s="1" t="n">
+        <v>0.1595001667737961</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-12T08:51:45Z</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>"What are the dimensions for d_model, d_k, d_v, and the number of attention heads (h) used in the Transformer base model?"</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>7</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G20" t="n">
+        <v>329</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2709</v>
+      </c>
+      <c r="I20" s="1" t="n">
+        <v>89.17050691244239</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>34485.33510044217</v>
+      </c>
+      <c r="L20" s="1" t="n">
+        <v>2121.531399898231</v>
+      </c>
+      <c r="M20" s="1" t="n">
+        <v>1033.575300127268</v>
+      </c>
+      <c r="N20" s="1" t="n">
+        <v>2121.531399898231</v>
+      </c>
+      <c r="O20" s="1" t="n">
+        <v>35518.91040056944</v>
+      </c>
+      <c r="P20" s="1" t="n">
+        <v>-33397.37900067121</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>458</v>
+      </c>
+      <c r="R20" t="n">
+        <v>187</v>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>The base Transformer model uses  
+* **d model = 512**  
+* **d k = d v = 64** (each head’s key and value vectors have dimension 64)  
+* **h = 8** attention heads  
+These values are given in the description of the multi‑head attention: “we employ **h = 8** parallel attention layers … for each of these we use **d_k = d_v = d_model / h = 64**.” Since h = 8, d_model = 8 × 64 = 512.</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>The provided context only states that the model uses **8 attention heads (h = 8)**. It does not give the specific values for **d_model**, **d_k**, or **d_v** for the Transformer base model. Therefore, the context does not contain enough information to answer those parts of the question.</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr"/>
+      <c r="V20" s="1" t="n"/>
+      <c r="W20" s="1" t="n"/>
+      <c r="X20" s="3" t="n"/>
+      <c r="Y20" s="3" t="n"/>
+      <c r="Z20" s="1" t="n"/>
+      <c r="AA20" s="1" t="n"/>
+      <c r="AB20" s="7" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE20" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF20" s="7" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="3" t="inlineStr">
+        <is>
+          <t>4,7,12,39,44,97</t>
+        </is>
+      </c>
+      <c r="AI20" s="1" t="n">
+        <v>17195.30799984932</v>
+      </c>
+      <c r="AJ20" s="1" t="n">
+        <v>17275.29519982636</v>
+      </c>
+      <c r="AK20" s="1" t="n">
+        <v>0.1929998397827148</v>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-12T08:58:31Z</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>"What are the dimensions for d_model, d_k, d_v, and the number of attention heads (h) used in the Transformer base model?"</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2873</v>
+      </c>
+      <c r="H21" t="n">
+        <v>165</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>5.4312047399605</v>
+      </c>
+      <c r="J21" t="n">
+        <v>109</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>36599.03069958091</v>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>2093.542099930346</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>1464.439999312162</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>2093.542099930346</v>
+      </c>
+      <c r="O21" s="1" t="n">
+        <v>38063.47069889307</v>
+      </c>
+      <c r="P21" s="1" t="n">
+        <v>-35969.92859896272</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>458</v>
+      </c>
+      <c r="R21" t="n">
+        <v>315</v>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>The base Transformer model uses  
+* **d model = 512**  
+* **d k = d v = 64** (each head’s key and value vectors have dimension 64)  
+* **h = 8** attention heads  
+These values are given in the description of the multi‑head attention: “we employ **h = 8** parallel attention layers … for each of these we use **d_k = d_v = d_model / h = 64**.” Since h = 8, d_model = 8 × 64 = 512.</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>The base Transformer model uses  
+- **d model = 512** (the dimensionality of the input and output vectors of each layer)  
+- **h = 8** attention heads  
+- For each head, the projected key and value dimensions are **d k = d v = d model / h = 64**.</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr"/>
+      <c r="V21" s="1" t="n"/>
+      <c r="W21" s="1" t="n"/>
+      <c r="X21" s="3" t="n"/>
+      <c r="Y21" s="3" t="n"/>
+      <c r="Z21" s="1" t="n"/>
+      <c r="AA21" s="1" t="n"/>
+      <c r="AB21" s="7" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE21" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF21" s="7" t="n">
+        <v>0.8260000000000001</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH21" s="3" t="inlineStr">
+        <is>
+          <t>0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,118,119,120,121,122,123,124,125,126,127,128</t>
+        </is>
+      </c>
+      <c r="AI21" s="1" t="n">
+        <v>19096.48740012199</v>
+      </c>
+      <c r="AJ21" s="1" t="n">
+        <v>17477.91450005025</v>
+      </c>
+      <c r="AK21" s="1" t="n">
+        <v>0.1600999385118484</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-13T03:33:30Z</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>"What were Apple's total net sales and net income for the three months ended June 29, 2024, compared to the three months ended July 1, 2023?</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G22" t="n">
+        <v>628</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2410</v>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>79.32850559578671</v>
+      </c>
+      <c r="J22" t="n">
+        <v>18</v>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>35325.85899997503</v>
+      </c>
+      <c r="L22" s="1" t="n">
+        <v>1414.723999798298</v>
+      </c>
+      <c r="M22" s="1" t="n">
+        <v>1132.796599529684</v>
+      </c>
+      <c r="N22" s="1" t="n">
+        <v>1414.723999798298</v>
+      </c>
+      <c r="O22" s="1" t="n">
+        <v>36458.65559950471</v>
+      </c>
+      <c r="P22" s="1" t="n">
+        <v>-35043.93159970641</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>158</v>
+      </c>
+      <c r="R22" t="n">
+        <v>172</v>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain the figures for Apple’s total net sales or net income for the three months ended June 29 2024, nor for the three months ended July 1 2023. Therefore, the information needed to answer the question is not available in the given excerpt.</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain the figures for Apple’s total net sales or net income for the three months ended June 29 2024 or for the three months ended July 1 2023. Therefore, the information needed to answer the question is not available in the given excerpt.</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="inlineStr"/>
+      <c r="V22" s="1" t="n"/>
+      <c r="W22" s="1" t="n"/>
+      <c r="X22" s="3" t="n"/>
+      <c r="Y22" s="3" t="n"/>
+      <c r="Z22" s="1" t="n"/>
+      <c r="AA22" s="1" t="n"/>
+      <c r="AB22" s="7" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE22" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF22" s="7" t="n">
+        <v>0.8330000000000001</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="3" t="inlineStr">
+        <is>
+          <t>1,2,3,23,24,25,34,35,36,59,60,61,68,69,70,71,72,73</t>
+        </is>
+      </c>
+      <c r="AI22" s="1" t="n">
+        <v>16961.68980002403</v>
+      </c>
+      <c r="AJ22" s="1" t="n">
+        <v>18351.5583993867</v>
+      </c>
+      <c r="AK22" s="1" t="n">
+        <v>0.1456998288631439</v>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-13T03:40:19Z</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>What were Apple's total net sales and net income for the three months ended June 29, 2024, compared to the three months ended July 1, 2023?</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3037</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2965</v>
+      </c>
+      <c r="H23" t="n">
+        <v>72</v>
+      </c>
+      <c r="I23" s="1" t="n">
+        <v>2.37076061903194</v>
+      </c>
+      <c r="J23" t="n">
+        <v>96</v>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>33943.61170008779</v>
+      </c>
+      <c r="L23" s="1" t="n">
+        <v>1871.478799730539</v>
+      </c>
+      <c r="M23" s="1" t="n">
+        <v>1122.418300248682</v>
+      </c>
+      <c r="N23" s="1" t="n">
+        <v>1871.478799730539</v>
+      </c>
+      <c r="O23" s="1" t="n">
+        <v>35066.03000033647</v>
+      </c>
+      <c r="P23" s="1" t="n">
+        <v>-33194.55120060593</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>186</v>
+      </c>
+      <c r="R23" t="n">
+        <v>186</v>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain Apple’s total net sales or net income for the three months ended June 29 2024 or for the three months ended July 1 2023. Therefore, the information needed to answer the question is not available in the given excerpt.</t>
+        </is>
+      </c>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain the figures for Apple’s total net sales or net income for the three months ended June 29 2024 or for the three months ended July 1 2023. Therefore, the information needed to answer the question is not available in the given excerpt.</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr"/>
+      <c r="V23" s="1" t="n"/>
+      <c r="W23" s="1" t="n"/>
+      <c r="X23" s="3" t="n"/>
+      <c r="Y23" s="3" t="n"/>
+      <c r="Z23" s="1" t="n"/>
+      <c r="AA23" s="1" t="n"/>
+      <c r="AB23" s="7" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE23" s="7" t="n">
+        <v>0.08399999999999999</v>
+      </c>
+      <c r="AF23" s="7" t="n">
+        <v>0.831</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="3" t="inlineStr">
+        <is>
+          <t>0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,97,98,99,100,102,103,104,105,106</t>
+        </is>
+      </c>
+      <c r="AI23" s="1" t="n">
+        <v>17752.99800001085</v>
+      </c>
+      <c r="AJ23" s="1" t="n">
+        <v>16170.74729967862</v>
+      </c>
+      <c r="AK23" s="1" t="n">
+        <v>0.1120995730161667</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-13T03:46:06Z</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>What were Apple's total net sales and net income for the three months ended June 29, 2024, compared to the three months ended July 1, 2023</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2848</v>
+      </c>
+      <c r="H24" t="n">
+        <v>190</v>
+      </c>
+      <c r="I24" s="1" t="n">
+        <v>6.254114549045426</v>
+      </c>
+      <c r="J24" t="n">
+        <v>82</v>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>39082.33710005879</v>
+      </c>
+      <c r="L24" s="1" t="n">
+        <v>1313.393299467862</v>
+      </c>
+      <c r="M24" s="1" t="n">
+        <v>1122.464300133288</v>
+      </c>
+      <c r="N24" s="1" t="n">
+        <v>1313.393299467862</v>
+      </c>
+      <c r="O24" s="1" t="n">
+        <v>40204.80140019208</v>
+      </c>
+      <c r="P24" s="1" t="n">
+        <v>-38891.40810072422</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>138</v>
+      </c>
+      <c r="R24" t="n">
+        <v>179</v>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain any information about Apple’s total net sales or net income for the three months ended June 29 2024 or for the three months ended July 1 2023. Therefore, the answer cannot be derived from the given material.</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>The provided context does not contain information about Apple’s total net sales or net income for the three months ended June 29 2024 or for the three months ended July 1 2023. Therefore, I cannot answer the question based on the given material.</t>
+        </is>
+      </c>
+      <c r="U24" s="3" t="inlineStr"/>
+      <c r="V24" s="1" t="n"/>
+      <c r="W24" s="1" t="n"/>
+      <c r="X24" s="3" t="n"/>
+      <c r="Y24" s="3" t="n"/>
+      <c r="Z24" s="1" t="n"/>
+      <c r="AA24" s="1" t="n"/>
+      <c r="AB24" s="7" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="AE24" s="7" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="AF24" s="7" t="n">
+        <v>0.8330000000000001</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="3" t="inlineStr">
+        <is>
+          <t>0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,32,33,34,35,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,83,84,85,86,87,88,90,91,92,93,94,95,96,97,98,99,100</t>
+        </is>
+      </c>
+      <c r="AI24" s="1" t="n">
+        <v>20634.31399967521</v>
+      </c>
+      <c r="AJ24" s="1" t="n">
+        <v>18429.93539944291</v>
+      </c>
+      <c r="AK24" s="1" t="n">
+        <v>0.1368001103401184</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AK16"/>
+  <autoFilter ref="A1:AK24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>